<commit_message>
Improved legend display on plot_inputs
</commit_message>
<xml_diff>
--- a/inputs/seep/xslope_lost_lake.xlsx
+++ b/inputs/seep/xslope_lost_lake.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/njones/python_projects/xslope/inputs/seep/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E2585C4-3584-B047-81B2-B2814A79AF40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A05A6C93-5373-2144-A77B-39755506909E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4360" yWindow="2980" windowWidth="25780" windowHeight="22880" activeTab="3" xr2:uid="{BA54C293-CE08-6E4C-9212-B3317DAA148E}"/>
+    <workbookView xWindow="33060" yWindow="2600" windowWidth="25780" windowHeight="22880" activeTab="2" xr2:uid="{BA54C293-CE08-6E4C-9212-B3317DAA148E}"/>
   </bookViews>
   <sheets>
     <sheet name="main" sheetId="1" r:id="rId1"/>
@@ -56,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="248" uniqueCount="161">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="161">
   <si>
     <t>X</t>
   </si>
@@ -8866,18 +8866,10 @@
       <c r="A3" s="3">
         <v>1</v>
       </c>
-      <c r="B3" s="3">
-        <v>100</v>
-      </c>
-      <c r="C3" s="3">
-        <v>500</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="E3" s="3">
-        <v>197</v>
-      </c>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
       <c r="F3" s="3"/>
       <c r="G3" s="3"/>
       <c r="H3" s="3"/>
@@ -8892,18 +8884,10 @@
       <c r="A4" s="3">
         <v>2</v>
       </c>
-      <c r="B4" s="3">
-        <v>100</v>
-      </c>
-      <c r="C4" s="3">
-        <v>500</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="E4" s="3">
-        <v>182</v>
-      </c>
+      <c r="B4" s="3"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
       <c r="F4" s="3"/>
       <c r="G4" s="3"/>
       <c r="H4" s="3"/>

</xml_diff>

<commit_message>
fixed polygon creation issues for lost lake problem
</commit_message>
<xml_diff>
--- a/inputs/seep/xslope_lost_lake.xlsx
+++ b/inputs/seep/xslope_lost_lake.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/njones/python_projects/xslope/inputs/seep/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A05A6C93-5373-2144-A77B-39755506909E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F0FFBBA-2867-A94F-8800-D8698623DF87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="33060" yWindow="2600" windowWidth="25780" windowHeight="22880" activeTab="2" xr2:uid="{BA54C293-CE08-6E4C-9212-B3317DAA148E}"/>
+    <workbookView xWindow="38380" yWindow="2180" windowWidth="25780" windowHeight="22880" activeTab="3" xr2:uid="{BA54C293-CE08-6E4C-9212-B3317DAA148E}"/>
   </bookViews>
   <sheets>
     <sheet name="main" sheetId="1" r:id="rId1"/>
@@ -7968,7 +7968,7 @@
         <v>0</v>
       </c>
       <c r="U4" s="3">
-        <v>1E-3</v>
+        <v>1E-4</v>
       </c>
       <c r="V4" s="3">
         <v>-1</v>
@@ -8008,7 +8008,7 @@
         <v>0</v>
       </c>
       <c r="U5" s="3">
-        <v>1E-3</v>
+        <v>1E-4</v>
       </c>
       <c r="V5" s="3">
         <v>-1</v>
@@ -8048,7 +8048,7 @@
         <v>0</v>
       </c>
       <c r="U6" s="3">
-        <v>1E-3</v>
+        <v>1E-4</v>
       </c>
       <c r="V6" s="3">
         <v>-1</v>
@@ -8088,7 +8088,7 @@
         <v>0</v>
       </c>
       <c r="U7" s="3">
-        <v>1E-3</v>
+        <v>1E-4</v>
       </c>
       <c r="V7" s="3">
         <v>-1</v>
@@ -8127,8 +8127,8 @@
       <c r="T8" s="16">
         <v>0</v>
       </c>
-      <c r="U8" s="17">
-        <v>1E-3</v>
+      <c r="U8" s="3">
+        <v>1E-4</v>
       </c>
       <c r="V8" s="17">
         <v>-1</v>
@@ -8167,8 +8167,8 @@
       <c r="T9" s="16">
         <v>0</v>
       </c>
-      <c r="U9" s="17">
-        <v>1E-3</v>
+      <c r="U9" s="3">
+        <v>1E-4</v>
       </c>
       <c r="V9" s="17">
         <v>-1</v>
@@ -8207,8 +8207,8 @@
       <c r="T10" s="16">
         <v>0</v>
       </c>
-      <c r="U10" s="17">
-        <v>1E-3</v>
+      <c r="U10" s="3">
+        <v>1E-4</v>
       </c>
       <c r="V10" s="17">
         <v>-1</v>
@@ -8247,8 +8247,8 @@
       <c r="T11" s="16">
         <v>0</v>
       </c>
-      <c r="U11" s="17">
-        <v>1E-3</v>
+      <c r="U11" s="3">
+        <v>1E-4</v>
       </c>
       <c r="V11" s="17">
         <v>-1</v>
@@ -8287,8 +8287,8 @@
       <c r="T12" s="16">
         <v>0</v>
       </c>
-      <c r="U12" s="17">
-        <v>1E-3</v>
+      <c r="U12" s="3">
+        <v>1E-4</v>
       </c>
       <c r="V12" s="17">
         <v>-1</v>
@@ -8327,8 +8327,8 @@
       <c r="T13" s="16">
         <v>0</v>
       </c>
-      <c r="U13" s="17">
-        <v>1E-3</v>
+      <c r="U13" s="3">
+        <v>1E-4</v>
       </c>
       <c r="V13" s="17">
         <v>-1</v>
@@ -8367,8 +8367,8 @@
       <c r="T14" s="16">
         <v>0</v>
       </c>
-      <c r="U14" s="17">
-        <v>1E-3</v>
+      <c r="U14" s="3">
+        <v>1E-4</v>
       </c>
       <c r="V14" s="17">
         <v>-1</v>
@@ -8407,8 +8407,8 @@
       <c r="T15" s="16">
         <v>0</v>
       </c>
-      <c r="U15" s="17">
-        <v>1E-3</v>
+      <c r="U15" s="3">
+        <v>1E-4</v>
       </c>
       <c r="V15" s="17">
         <v>-1</v>

</xml_diff>